<commit_message>
Create database tables inside the features that first need them
Replaces the upfront database task with a per-feature Database column
and adds a Schema sheet listing every table and column.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016VxfYAmeTkhYFto1GdTc34
</commit_message>
<xml_diff>
--- a/Store_Shield_Estimation.xlsx
+++ b/Store_Shield_Estimation.xlsx
@@ -9,6 +9,7 @@
   </bookViews>
   <sheets>
     <sheet name="Estimate" sheetId="1" state="visible" r:id="rId3"/>
+    <sheet name="Schema" sheetId="2" state="visible" r:id="rId4"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -20,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="89">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="268" uniqueCount="185">
   <si>
     <t xml:space="preserve">Store Shield - Estimate</t>
   </si>
@@ -34,6 +35,9 @@
     <t xml:space="preserve">Description</t>
   </si>
   <si>
+    <t xml:space="preserve">Database</t>
+  </si>
+  <si>
     <t xml:space="preserve">Hours</t>
   </si>
   <si>
@@ -46,10 +50,7 @@
     <t xml:space="preserve">Make the Shopify app and run it</t>
   </si>
   <si>
-    <t xml:space="preserve">Database</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tables to save all data</t>
+    <t xml:space="preserve">NEW sessions (comes with Shopify template): Shopify login sessions</t>
   </si>
   <si>
     <t xml:space="preserve">Default settings</t>
@@ -58,12 +59,18 @@
     <t xml:space="preserve">Starting scores and limits</t>
   </si>
   <si>
+    <t xml:space="preserve">NEW settings: shop, bot_mode, fraud_mode, bot cut-offs, fraud cut-offs, bot_points, fraud_points</t>
+  </si>
+  <si>
     <t xml:space="preserve">Test store</t>
   </si>
   <si>
     <t xml:space="preserve">Sample products and test payments</t>
   </si>
   <si>
+    <t xml:space="preserve">-</t>
+  </si>
+  <si>
     <t xml:space="preserve">2. Bot Check</t>
   </si>
   <si>
@@ -91,12 +98,18 @@
     <t xml:space="preserve">Add up points, score 0-100</t>
   </si>
   <si>
+    <t xml:space="preserve">- (page-burst counter kept in memory)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Visitor log</t>
   </si>
   <si>
     <t xml:space="preserve">Save every visit and score</t>
   </si>
   <si>
+    <t xml:space="preserve">NEW visits: shop, device_id, ip, page, score, reasons, action, created_at</t>
+  </si>
+  <si>
     <t xml:space="preserve">Challenge &amp; block</t>
   </si>
   <si>
@@ -109,6 +122,9 @@
     <t xml:space="preserve">Attach bot score to the order</t>
   </si>
   <si>
+    <t xml:space="preserve">- (stored on the Shopify cart)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Spy-tool check (optional)</t>
   </si>
   <si>
@@ -130,6 +146,9 @@
     <t xml:space="preserve">Known fraudster = high risk</t>
   </si>
   <si>
+    <t xml:space="preserve">NEW fraud_list: shop, type (email/phone/address/card/device/ip), value, order_id, created_at</t>
+  </si>
+  <si>
     <t xml:space="preserve">Shopify risk</t>
   </si>
   <si>
@@ -154,30 +173,45 @@
     <t xml:space="preserve">Add up points, decide action</t>
   </si>
   <si>
+    <t xml:space="preserve">NEW order_checks: shop, order_id, customer_id, email, phone, ip, billing, shipping, card_last4, card_brand, device_id, bot_score, score, reasons, decision, status, created_at</t>
+  </si>
+  <si>
     <t xml:space="preserve">Hold order</t>
   </si>
   <si>
     <t xml:space="preserve">Stop shipping until reviewed</t>
   </si>
   <si>
+    <t xml:space="preserve">- (updates order_checks.status)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Auto-cancel</t>
   </si>
   <si>
     <t xml:space="preserve">Cancel, refund, restock, email</t>
   </si>
   <si>
+    <t xml:space="preserve">CHANGE settings: + auto_cancel (on/off)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Good signs</t>
   </si>
   <si>
     <t xml:space="preserve">Loyal customers get lower score</t>
   </si>
   <si>
+    <t xml:space="preserve">- (reads past order_checks)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Risky products</t>
   </si>
   <si>
     <t xml:space="preserve">Limits on easy-to-resell items</t>
   </si>
   <si>
+    <t xml:space="preserve">CHANGE settings: + risky_categories, risky_limits</t>
+  </si>
+  <si>
     <t xml:space="preserve">Failed payments (optional)</t>
   </si>
   <si>
@@ -205,30 +239,45 @@
     <t xml:space="preserve">Held orders with approve/cancel</t>
   </si>
   <si>
+    <t xml:space="preserve">NEW staff_actions: shop, action, target, note, created_at</t>
+  </si>
+  <si>
     <t xml:space="preserve">Bot activity</t>
   </si>
   <si>
     <t xml:space="preserve">Blocked visitors with unblock</t>
   </si>
   <si>
+    <t xml:space="preserve">NEW trust_list: shop, type (device/customer/email/ip), value, reason, expires_at, created_at</t>
+  </si>
+  <si>
     <t xml:space="preserve">Settings</t>
   </si>
   <si>
     <t xml:space="preserve">Change scores, limits, on/off</t>
   </si>
   <si>
+    <t xml:space="preserve">- (edits settings)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Overview</t>
   </si>
   <si>
     <t xml:space="preserve">Today's numbers at a glance</t>
   </si>
   <si>
+    <t xml:space="preserve">- (counts visits, order_checks)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Activity log</t>
   </si>
   <si>
     <t xml:space="preserve">History of actions, with undo</t>
   </si>
   <si>
+    <t xml:space="preserve">- (reads visits, order_checks, staff_actions)</t>
+  </si>
+  <si>
     <t xml:space="preserve">5. Fraud Tagging</t>
   </si>
   <si>
@@ -238,18 +287,27 @@
     <t xml:space="preserve">Tag customer, save to fraud list</t>
   </si>
   <si>
+    <t xml:space="preserve">- (writes fraud_list, updates order_checks.status)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Catch returning fraudster</t>
   </si>
   <si>
     <t xml:space="preserve">Flag their device next visit</t>
   </si>
   <si>
+    <t xml:space="preserve">- (bot score reads fraud_list)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Trust &amp; fraud lists</t>
   </si>
   <si>
     <t xml:space="preserve">Trust or remove customers</t>
   </si>
   <si>
+    <t xml:space="preserve">- (edits trust_list, fraud_list)</t>
+  </si>
+  <si>
     <t xml:space="preserve">6. Testing &amp; Launch</t>
   </si>
   <si>
@@ -277,6 +335,9 @@
     <t xml:space="preserve">Put the app online</t>
   </si>
   <si>
+    <t xml:space="preserve">Move from SQLite to Postgres</t>
+  </si>
+  <si>
     <t xml:space="preserve">Fix bugs</t>
   </si>
   <si>
@@ -287,6 +348,234 @@
   </si>
   <si>
     <t xml:space="preserve">Hours are hands-on hours building with Claude Code. Optional items can be skipped to save 3 hours.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Database tables</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Table</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Created in</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Column</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Type</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Meaning</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sessions</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(from Shopify template)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Shopify login sessions</t>
+  </si>
+  <si>
+    <t xml:space="preserve">settings</t>
+  </si>
+  <si>
+    <t xml:space="preserve">shop</t>
+  </si>
+  <si>
+    <t xml:space="preserve">text, key</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Store domain</t>
+  </si>
+  <si>
+    <t xml:space="preserve">bot_mode / fraud_mode</t>
+  </si>
+  <si>
+    <t xml:space="preserve">text</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test or live</t>
+  </si>
+  <si>
+    <t xml:space="preserve">bot_low_max / bot_medium_max</t>
+  </si>
+  <si>
+    <t xml:space="preserve">int</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bot score cut-offs (30 / 70)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fraud_low_max / fraud_medium_max</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fraud score cut-offs (30 / 70)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">bot_points / fraud_points</t>
+  </si>
+  <si>
+    <t xml:space="preserve">json</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Points per factor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">auto_cancel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">bool</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Added in Auto-cancel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">risky_categories / risky_limits</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Added in Risky products</t>
+  </si>
+  <si>
+    <t xml:space="preserve">visits</t>
+  </si>
+  <si>
+    <t xml:space="preserve">id</t>
+  </si>
+  <si>
+    <t xml:space="preserve">int, key</t>
+  </si>
+  <si>
+    <t xml:space="preserve">device_id</t>
+  </si>
+  <si>
+    <t xml:space="preserve">From the visitor cookie</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ip</t>
+  </si>
+  <si>
+    <t xml:space="preserve">page</t>
+  </si>
+  <si>
+    <t xml:space="preserve">score</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0-100</t>
+  </si>
+  <si>
+    <t xml:space="preserve">reasons</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Which checks added points</t>
+  </si>
+  <si>
+    <t xml:space="preserve">action</t>
+  </si>
+  <si>
+    <t xml:space="preserve">allow / challenge / block</t>
+  </si>
+  <si>
+    <t xml:space="preserve">created_at</t>
+  </si>
+  <si>
+    <t xml:space="preserve">datetime</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fraud_list</t>
+  </si>
+  <si>
+    <t xml:space="preserve">type</t>
+  </si>
+  <si>
+    <t xml:space="preserve">email / phone / address / card / device / ip</t>
+  </si>
+  <si>
+    <t xml:space="preserve">value</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The flagged value</t>
+  </si>
+  <si>
+    <t xml:space="preserve">order_id</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Order that confirmed the fraud</t>
+  </si>
+  <si>
+    <t xml:space="preserve">order_checks</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Shopify order</t>
+  </si>
+  <si>
+    <t xml:space="preserve">customer_id</t>
+  </si>
+  <si>
+    <t xml:space="preserve">email / phone / ip</t>
+  </si>
+  <si>
+    <t xml:space="preserve">billing / shipping</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Addresses</t>
+  </si>
+  <si>
+    <t xml:space="preserve">card_last4 / card_brand</t>
+  </si>
+  <si>
+    <t xml:space="preserve">device_id / bot_score</t>
+  </si>
+  <si>
+    <t xml:space="preserve">text / int</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Carried from the visit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Plain-English reasons</t>
+  </si>
+  <si>
+    <t xml:space="preserve">decision</t>
+  </si>
+  <si>
+    <t xml:space="preserve">approve / hold / cancel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">status</t>
+  </si>
+  <si>
+    <t xml:space="preserve">approved / held / cancelled / fraud</t>
+  </si>
+  <si>
+    <t xml:space="preserve">staff_actions</t>
+  </si>
+  <si>
+    <t xml:space="preserve">approve / cancel / unblock / mark_fraud / remove / reinstate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">target</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Order, device or list entry</t>
+  </si>
+  <si>
+    <t xml:space="preserve">note</t>
+  </si>
+  <si>
+    <t xml:space="preserve">trust_list</t>
+  </si>
+  <si>
+    <t xml:space="preserve">device / customer / email / ip</t>
+  </si>
+  <si>
+    <t xml:space="preserve">reason</t>
+  </si>
+  <si>
+    <t xml:space="preserve">expires_at</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Empty = forever</t>
   </si>
 </sst>
 </file>
@@ -425,7 +714,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="13">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -443,15 +732,15 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="165" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="165" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
@@ -459,10 +748,22 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="165" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -718,13 +1019,14 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D50"/>
+  <dimension ref="A1:E49"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="20"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="28"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="40"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="36"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="60"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="9"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -745,544 +1047,1318 @@
       <c r="D3" s="2" t="s">
         <v>4</v>
       </c>
+      <c r="E3" s="2" t="s">
+        <v>5</v>
+      </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B4" s="3"/>
       <c r="C4" s="3"/>
-      <c r="D4" s="4" t="n">
-        <f aca="false">SUM(D5:D8)</f>
-        <v>5</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D4" s="3"/>
+      <c r="E4" s="4" t="n">
+        <f aca="false">SUM(E5:E7)</f>
+        <v>3.75</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="5"/>
       <c r="B5" s="5" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="D5" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="E5" s="6" t="n">
         <v>2</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="5"/>
       <c r="B6" s="5" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="D6" s="6" t="n">
-        <v>1.5</v>
+        <v>11</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="E6" s="6" t="n">
+        <v>0.75</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="5"/>
       <c r="B7" s="5" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="D7" s="6" t="n">
-        <v>0.5</v>
+        <v>14</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="E7" s="6" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="5"/>
-      <c r="B8" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="C8" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="D8" s="6" t="n">
-        <v>1</v>
+      <c r="A8" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B8" s="3"/>
+      <c r="C8" s="3"/>
+      <c r="D8" s="3"/>
+      <c r="E8" s="4" t="n">
+        <f aca="false">SUM(E9:E16)</f>
+        <v>13.75</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="B9" s="3"/>
-      <c r="C9" s="3"/>
-      <c r="D9" s="4" t="n">
-        <f aca="false">SUM(D10:D17)</f>
-        <v>13.5</v>
+      <c r="A9" s="5"/>
+      <c r="B9" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="E9" s="6" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="5"/>
       <c r="B10" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="D10" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="C10" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="D10" s="6" t="n">
-        <v>2</v>
+      <c r="E10" s="6" t="n">
+        <v>1.5</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="5"/>
       <c r="B11" s="5" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="D11" s="6" t="n">
-        <v>1.5</v>
+        <v>22</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="E11" s="6" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="5"/>
       <c r="B12" s="5" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="D12" s="6" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>24</v>
+      </c>
+      <c r="D12" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="E12" s="6" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="5"/>
       <c r="B13" s="5" t="s">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="D13" s="6" t="n">
-        <v>3</v>
+        <v>27</v>
+      </c>
+      <c r="D13" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="E13" s="6" t="n">
+        <v>0.75</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="5"/>
       <c r="B14" s="5" t="s">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="D14" s="6" t="n">
-        <v>0.5</v>
+        <v>30</v>
+      </c>
+      <c r="D14" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="E14" s="6" t="n">
+        <v>2.5</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="5"/>
       <c r="B15" s="5" t="s">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="D15" s="6" t="n">
-        <v>2.5</v>
+        <v>32</v>
+      </c>
+      <c r="D15" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="E15" s="6" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="5"/>
       <c r="B16" s="5" t="s">
-        <v>27</v>
+        <v>34</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="D16" s="6" t="n">
+        <v>35</v>
+      </c>
+      <c r="D16" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="E16" s="6" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="5"/>
-      <c r="B17" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="C17" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="D17" s="6" t="n">
-        <v>1</v>
+      <c r="A17" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="B17" s="3"/>
+      <c r="C17" s="3"/>
+      <c r="D17" s="3"/>
+      <c r="E17" s="4" t="n">
+        <f aca="false">SUM(E18:E29)</f>
+        <v>15.5</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="B18" s="3"/>
-      <c r="C18" s="3"/>
-      <c r="D18" s="4" t="n">
-        <f aca="false">SUM(D19:D30)</f>
+      <c r="A18" s="5"/>
+      <c r="B18" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="C18" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="D18" s="5" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E18" s="6" t="n">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="5"/>
       <c r="B19" s="5" t="s">
-        <v>32</v>
+        <v>39</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="D19" s="6" t="n">
-        <v>1.5</v>
+        <v>40</v>
+      </c>
+      <c r="D19" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="E19" s="6" t="n">
+        <v>1.25</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="5"/>
       <c r="B20" s="5" t="s">
-        <v>34</v>
+        <v>42</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>35</v>
-      </c>
-      <c r="D20" s="6" t="n">
+        <v>43</v>
+      </c>
+      <c r="D20" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="E20" s="6" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="5"/>
       <c r="B21" s="5" t="s">
-        <v>36</v>
+        <v>44</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>37</v>
-      </c>
-      <c r="D21" s="6" t="n">
-        <v>1</v>
+        <v>45</v>
+      </c>
+      <c r="D21" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="E21" s="6" t="n">
+        <v>2.5</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="5"/>
       <c r="B22" s="5" t="s">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>39</v>
-      </c>
-      <c r="D22" s="6" t="n">
-        <v>2.5</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>47</v>
+      </c>
+      <c r="D22" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="E22" s="6" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="5"/>
       <c r="B23" s="5" t="s">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>41</v>
-      </c>
-      <c r="D23" s="6" t="n">
-        <v>0.5</v>
+        <v>49</v>
+      </c>
+      <c r="D23" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="E23" s="6" t="n">
+        <v>1.25</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="5"/>
       <c r="B24" s="5" t="s">
-        <v>42</v>
+        <v>51</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>43</v>
-      </c>
-      <c r="D24" s="6" t="n">
-        <v>1</v>
+        <v>52</v>
+      </c>
+      <c r="D24" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="E24" s="6" t="n">
+        <v>1.5</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="5"/>
       <c r="B25" s="5" t="s">
-        <v>44</v>
+        <v>54</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>45</v>
-      </c>
-      <c r="D25" s="6" t="n">
+        <v>55</v>
+      </c>
+      <c r="D25" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="E25" s="6" t="n">
         <v>1.5</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="5"/>
       <c r="B26" s="5" t="s">
-        <v>46</v>
+        <v>57</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="D26" s="6" t="n">
+        <v>58</v>
+      </c>
+      <c r="D26" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="E26" s="6" t="n">
         <v>1.5</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="5"/>
       <c r="B27" s="5" t="s">
-        <v>48</v>
+        <v>60</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>49</v>
-      </c>
-      <c r="D27" s="6" t="n">
-        <v>1.5</v>
+        <v>61</v>
+      </c>
+      <c r="D27" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="E27" s="6" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="5"/>
       <c r="B28" s="5" t="s">
-        <v>50</v>
+        <v>63</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="D28" s="6" t="n">
+        <v>64</v>
+      </c>
+      <c r="D28" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="E28" s="6" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="5"/>
       <c r="B29" s="5" t="s">
-        <v>52</v>
+        <v>65</v>
       </c>
       <c r="C29" s="5" t="s">
-        <v>53</v>
-      </c>
-      <c r="D29" s="6" t="n">
+        <v>66</v>
+      </c>
+      <c r="D29" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="E29" s="6" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="5"/>
-      <c r="B30" s="5" t="s">
-        <v>54</v>
-      </c>
-      <c r="C30" s="5" t="s">
-        <v>55</v>
-      </c>
-      <c r="D30" s="6" t="n">
-        <v>1</v>
+      <c r="A30" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="B30" s="3"/>
+      <c r="C30" s="3"/>
+      <c r="D30" s="3"/>
+      <c r="E30" s="4" t="n">
+        <f aca="false">SUM(E31:E36)</f>
+        <v>11</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="B31" s="3"/>
-      <c r="C31" s="3"/>
-      <c r="D31" s="4" t="n">
-        <f aca="false">SUM(D32:D37)</f>
-        <v>10.5</v>
+      <c r="A31" s="5"/>
+      <c r="B31" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="C31" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="D31" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="E31" s="6" t="n">
+        <v>0.5</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="5"/>
       <c r="B32" s="5" t="s">
-        <v>57</v>
+        <v>70</v>
       </c>
       <c r="C32" s="5" t="s">
-        <v>58</v>
-      </c>
-      <c r="D32" s="6" t="n">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>71</v>
+      </c>
+      <c r="D32" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="E32" s="6" t="n">
+        <v>3.25</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="5"/>
       <c r="B33" s="5" t="s">
-        <v>59</v>
+        <v>73</v>
       </c>
       <c r="C33" s="5" t="s">
-        <v>60</v>
-      </c>
-      <c r="D33" s="6" t="n">
-        <v>3</v>
+        <v>74</v>
+      </c>
+      <c r="D33" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="E33" s="6" t="n">
+        <v>1.75</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="5"/>
       <c r="B34" s="5" t="s">
-        <v>61</v>
+        <v>76</v>
       </c>
       <c r="C34" s="5" t="s">
-        <v>62</v>
-      </c>
-      <c r="D34" s="6" t="n">
-        <v>1.5</v>
+        <v>77</v>
+      </c>
+      <c r="D34" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="E34" s="6" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="5"/>
       <c r="B35" s="5" t="s">
-        <v>63</v>
+        <v>79</v>
       </c>
       <c r="C35" s="5" t="s">
-        <v>64</v>
-      </c>
-      <c r="D35" s="6" t="n">
-        <v>2</v>
+        <v>80</v>
+      </c>
+      <c r="D35" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="E35" s="6" t="n">
+        <v>1.5</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="5"/>
       <c r="B36" s="5" t="s">
-        <v>65</v>
+        <v>82</v>
       </c>
       <c r="C36" s="5" t="s">
-        <v>66</v>
-      </c>
-      <c r="D36" s="6" t="n">
+        <v>83</v>
+      </c>
+      <c r="D36" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="E36" s="6" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="B37" s="3"/>
+      <c r="C37" s="3"/>
+      <c r="D37" s="3"/>
+      <c r="E37" s="4" t="n">
+        <f aca="false">SUM(E38:E40)</f>
+        <v>3.5</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="5"/>
+      <c r="B38" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="C38" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="D38" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="E38" s="6" t="n">
         <v>1.5</v>
-      </c>
-    </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="5"/>
-      <c r="B37" s="5" t="s">
-        <v>67</v>
-      </c>
-      <c r="C37" s="5" t="s">
-        <v>68</v>
-      </c>
-      <c r="D37" s="6" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="3" t="s">
-        <v>69</v>
-      </c>
-      <c r="B38" s="3"/>
-      <c r="C38" s="3"/>
-      <c r="D38" s="4" t="n">
-        <f aca="false">SUM(D39:D41)</f>
-        <v>3.5</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="5"/>
       <c r="B39" s="5" t="s">
-        <v>70</v>
+        <v>89</v>
       </c>
       <c r="C39" s="5" t="s">
-        <v>71</v>
-      </c>
-      <c r="D39" s="6" t="n">
-        <v>1.5</v>
+        <v>90</v>
+      </c>
+      <c r="D39" s="5" t="s">
+        <v>91</v>
+      </c>
+      <c r="E39" s="6" t="n">
+        <v>0.5</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="5"/>
       <c r="B40" s="5" t="s">
-        <v>72</v>
+        <v>92</v>
       </c>
       <c r="C40" s="5" t="s">
-        <v>73</v>
-      </c>
-      <c r="D40" s="6" t="n">
-        <v>0.5</v>
+        <v>93</v>
+      </c>
+      <c r="D40" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="E40" s="6" t="n">
+        <v>1.5</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="5"/>
-      <c r="B41" s="5" t="s">
-        <v>74</v>
-      </c>
-      <c r="C41" s="5" t="s">
-        <v>75</v>
-      </c>
-      <c r="D41" s="6" t="n">
+      <c r="A41" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="B41" s="3"/>
+      <c r="C41" s="3"/>
+      <c r="D41" s="3"/>
+      <c r="E41" s="4" t="n">
+        <f aca="false">SUM(E42:E46)</f>
+        <v>9</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="5"/>
+      <c r="B42" s="5" t="s">
+        <v>96</v>
+      </c>
+      <c r="C42" s="5" t="s">
+        <v>97</v>
+      </c>
+      <c r="D42" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="E42" s="6" t="n">
         <v>1.5</v>
-      </c>
-    </row>
-    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="3" t="s">
-        <v>76</v>
-      </c>
-      <c r="B42" s="3"/>
-      <c r="C42" s="3"/>
-      <c r="D42" s="4" t="n">
-        <f aca="false">SUM(D43:D47)</f>
-        <v>9</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="5"/>
       <c r="B43" s="5" t="s">
-        <v>77</v>
+        <v>98</v>
       </c>
       <c r="C43" s="5" t="s">
-        <v>78</v>
-      </c>
-      <c r="D43" s="6" t="n">
+        <v>99</v>
+      </c>
+      <c r="D43" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="E43" s="6" t="n">
         <v>1.5</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="5"/>
       <c r="B44" s="5" t="s">
-        <v>79</v>
+        <v>100</v>
       </c>
       <c r="C44" s="5" t="s">
-        <v>80</v>
-      </c>
-      <c r="D44" s="6" t="n">
-        <v>1.5</v>
+        <v>101</v>
+      </c>
+      <c r="D44" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="E44" s="6" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="5"/>
       <c r="B45" s="5" t="s">
-        <v>81</v>
+        <v>102</v>
       </c>
       <c r="C45" s="5" t="s">
-        <v>82</v>
-      </c>
-      <c r="D45" s="6" t="n">
-        <v>1</v>
+        <v>103</v>
+      </c>
+      <c r="D45" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="E45" s="6" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="5"/>
       <c r="B46" s="5" t="s">
-        <v>83</v>
+        <v>105</v>
       </c>
       <c r="C46" s="5" t="s">
-        <v>84</v>
-      </c>
-      <c r="D46" s="6" t="n">
-        <v>2</v>
+        <v>106</v>
+      </c>
+      <c r="D46" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="E46" s="6" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="5"/>
-      <c r="B47" s="5" t="s">
-        <v>85</v>
-      </c>
-      <c r="C47" s="5" t="s">
-        <v>86</v>
-      </c>
-      <c r="D47" s="6" t="n">
-        <v>3</v>
-      </c>
+      <c r="A47" s="7" t="s">
+        <v>107</v>
+      </c>
+      <c r="B47" s="7"/>
+      <c r="C47" s="7"/>
+      <c r="D47" s="7"/>
+      <c r="E47" s="8" t="n">
+        <f aca="false">E4+E8+E17+E30+E37+E41</f>
+        <v>56.5</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="9" t="s">
+        <v>108</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:E52"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="32"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="48"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="10" t="s">
+        <v>110</v>
+      </c>
+      <c r="B3" s="10" t="s">
+        <v>111</v>
+      </c>
+      <c r="C3" s="10" t="s">
+        <v>112</v>
+      </c>
+      <c r="D3" s="10" t="s">
+        <v>113</v>
+      </c>
+      <c r="E3" s="10" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C4" s="11" t="s">
+        <v>116</v>
+      </c>
+      <c r="D4" s="11"/>
+      <c r="E4" s="11" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C5" s="11" t="s">
+        <v>119</v>
+      </c>
+      <c r="D5" s="11" t="s">
+        <v>120</v>
+      </c>
+      <c r="E5" s="11" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="12"/>
+      <c r="B6" s="12"/>
+      <c r="C6" s="12" t="s">
+        <v>122</v>
+      </c>
+      <c r="D6" s="12" t="s">
+        <v>123</v>
+      </c>
+      <c r="E6" s="12" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="12"/>
+      <c r="B7" s="12"/>
+      <c r="C7" s="12" t="s">
+        <v>125</v>
+      </c>
+      <c r="D7" s="12" t="s">
+        <v>126</v>
+      </c>
+      <c r="E7" s="12" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="12"/>
+      <c r="B8" s="12"/>
+      <c r="C8" s="12" t="s">
+        <v>128</v>
+      </c>
+      <c r="D8" s="12" t="s">
+        <v>126</v>
+      </c>
+      <c r="E8" s="12" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="12"/>
+      <c r="B9" s="12"/>
+      <c r="C9" s="12" t="s">
+        <v>130</v>
+      </c>
+      <c r="D9" s="12" t="s">
+        <v>131</v>
+      </c>
+      <c r="E9" s="12" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="12"/>
+      <c r="B10" s="12"/>
+      <c r="C10" s="12" t="s">
+        <v>133</v>
+      </c>
+      <c r="D10" s="12" t="s">
+        <v>134</v>
+      </c>
+      <c r="E10" s="12" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="12"/>
+      <c r="B11" s="12"/>
+      <c r="C11" s="12" t="s">
+        <v>136</v>
+      </c>
+      <c r="D11" s="12" t="s">
+        <v>131</v>
+      </c>
+      <c r="E11" s="12" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="3" t="s">
+        <v>138</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="C12" s="11" t="s">
+        <v>139</v>
+      </c>
+      <c r="D12" s="11" t="s">
+        <v>140</v>
+      </c>
+      <c r="E12" s="11"/>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="12"/>
+      <c r="B13" s="12"/>
+      <c r="C13" s="12" t="s">
+        <v>119</v>
+      </c>
+      <c r="D13" s="12" t="s">
+        <v>123</v>
+      </c>
+      <c r="E13" s="12"/>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="12"/>
+      <c r="B14" s="12"/>
+      <c r="C14" s="12" t="s">
+        <v>141</v>
+      </c>
+      <c r="D14" s="12" t="s">
+        <v>123</v>
+      </c>
+      <c r="E14" s="12" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="12"/>
+      <c r="B15" s="12"/>
+      <c r="C15" s="12" t="s">
+        <v>143</v>
+      </c>
+      <c r="D15" s="12" t="s">
+        <v>123</v>
+      </c>
+      <c r="E15" s="12"/>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="12"/>
+      <c r="B16" s="12"/>
+      <c r="C16" s="12" t="s">
+        <v>144</v>
+      </c>
+      <c r="D16" s="12" t="s">
+        <v>123</v>
+      </c>
+      <c r="E16" s="12"/>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="12"/>
+      <c r="B17" s="12"/>
+      <c r="C17" s="12" t="s">
+        <v>145</v>
+      </c>
+      <c r="D17" s="12" t="s">
+        <v>126</v>
+      </c>
+      <c r="E17" s="12" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="12"/>
+      <c r="B18" s="12"/>
+      <c r="C18" s="12" t="s">
+        <v>147</v>
+      </c>
+      <c r="D18" s="12" t="s">
+        <v>131</v>
+      </c>
+      <c r="E18" s="12" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="12"/>
+      <c r="B19" s="12"/>
+      <c r="C19" s="12" t="s">
+        <v>149</v>
+      </c>
+      <c r="D19" s="12" t="s">
+        <v>123</v>
+      </c>
+      <c r="E19" s="12" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="12"/>
+      <c r="B20" s="12"/>
+      <c r="C20" s="12" t="s">
+        <v>151</v>
+      </c>
+      <c r="D20" s="12" t="s">
+        <v>152</v>
+      </c>
+      <c r="E20" s="12"/>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="C21" s="11" t="s">
+        <v>139</v>
+      </c>
+      <c r="D21" s="11" t="s">
+        <v>140</v>
+      </c>
+      <c r="E21" s="11"/>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="12"/>
+      <c r="B22" s="12"/>
+      <c r="C22" s="12" t="s">
+        <v>119</v>
+      </c>
+      <c r="D22" s="12" t="s">
+        <v>123</v>
+      </c>
+      <c r="E22" s="12"/>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="12"/>
+      <c r="B23" s="12"/>
+      <c r="C23" s="12" t="s">
+        <v>154</v>
+      </c>
+      <c r="D23" s="12" t="s">
+        <v>123</v>
+      </c>
+      <c r="E23" s="12" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="12"/>
+      <c r="B24" s="12"/>
+      <c r="C24" s="12" t="s">
+        <v>156</v>
+      </c>
+      <c r="D24" s="12" t="s">
+        <v>123</v>
+      </c>
+      <c r="E24" s="12" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="12"/>
+      <c r="B25" s="12"/>
+      <c r="C25" s="12" t="s">
+        <v>158</v>
+      </c>
+      <c r="D25" s="12" t="s">
+        <v>123</v>
+      </c>
+      <c r="E25" s="12" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="12"/>
+      <c r="B26" s="12"/>
+      <c r="C26" s="12" t="s">
+        <v>151</v>
+      </c>
+      <c r="D26" s="12" t="s">
+        <v>152</v>
+      </c>
+      <c r="E26" s="12"/>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="3" t="s">
+        <v>160</v>
+      </c>
+      <c r="B27" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="C27" s="11" t="s">
+        <v>139</v>
+      </c>
+      <c r="D27" s="11" t="s">
+        <v>140</v>
+      </c>
+      <c r="E27" s="11"/>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="12"/>
+      <c r="B28" s="12"/>
+      <c r="C28" s="12" t="s">
+        <v>119</v>
+      </c>
+      <c r="D28" s="12" t="s">
+        <v>123</v>
+      </c>
+      <c r="E28" s="12"/>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="12"/>
+      <c r="B29" s="12"/>
+      <c r="C29" s="12" t="s">
+        <v>158</v>
+      </c>
+      <c r="D29" s="12" t="s">
+        <v>123</v>
+      </c>
+      <c r="E29" s="12" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="12"/>
+      <c r="B30" s="12"/>
+      <c r="C30" s="12" t="s">
+        <v>162</v>
+      </c>
+      <c r="D30" s="12" t="s">
+        <v>123</v>
+      </c>
+      <c r="E30" s="12"/>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="12"/>
+      <c r="B31" s="12"/>
+      <c r="C31" s="12" t="s">
+        <v>163</v>
+      </c>
+      <c r="D31" s="12" t="s">
+        <v>123</v>
+      </c>
+      <c r="E31" s="12"/>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="12"/>
+      <c r="B32" s="12"/>
+      <c r="C32" s="12" t="s">
+        <v>164</v>
+      </c>
+      <c r="D32" s="12" t="s">
+        <v>123</v>
+      </c>
+      <c r="E32" s="12" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="12"/>
+      <c r="B33" s="12"/>
+      <c r="C33" s="12" t="s">
+        <v>166</v>
+      </c>
+      <c r="D33" s="12" t="s">
+        <v>123</v>
+      </c>
+      <c r="E33" s="12"/>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="12"/>
+      <c r="B34" s="12"/>
+      <c r="C34" s="12" t="s">
+        <v>167</v>
+      </c>
+      <c r="D34" s="12" t="s">
+        <v>168</v>
+      </c>
+      <c r="E34" s="12" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="12"/>
+      <c r="B35" s="12"/>
+      <c r="C35" s="12" t="s">
+        <v>145</v>
+      </c>
+      <c r="D35" s="12" t="s">
+        <v>126</v>
+      </c>
+      <c r="E35" s="12" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="12"/>
+      <c r="B36" s="12"/>
+      <c r="C36" s="12" t="s">
+        <v>147</v>
+      </c>
+      <c r="D36" s="12" t="s">
+        <v>131</v>
+      </c>
+      <c r="E36" s="12" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="12"/>
+      <c r="B37" s="12"/>
+      <c r="C37" s="12" t="s">
+        <v>171</v>
+      </c>
+      <c r="D37" s="12" t="s">
+        <v>123</v>
+      </c>
+      <c r="E37" s="12" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="12"/>
+      <c r="B38" s="12"/>
+      <c r="C38" s="12" t="s">
+        <v>173</v>
+      </c>
+      <c r="D38" s="12" t="s">
+        <v>123</v>
+      </c>
+      <c r="E38" s="12" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="12"/>
+      <c r="B39" s="12"/>
+      <c r="C39" s="12" t="s">
+        <v>151</v>
+      </c>
+      <c r="D39" s="12" t="s">
+        <v>152</v>
+      </c>
+      <c r="E39" s="12"/>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="3" t="s">
+        <v>175</v>
+      </c>
+      <c r="B40" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="C40" s="11" t="s">
+        <v>139</v>
+      </c>
+      <c r="D40" s="11" t="s">
+        <v>140</v>
+      </c>
+      <c r="E40" s="11"/>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="12"/>
+      <c r="B41" s="12"/>
+      <c r="C41" s="12" t="s">
+        <v>119</v>
+      </c>
+      <c r="D41" s="12" t="s">
+        <v>123</v>
+      </c>
+      <c r="E41" s="12"/>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="12"/>
+      <c r="B42" s="12"/>
+      <c r="C42" s="12" t="s">
+        <v>149</v>
+      </c>
+      <c r="D42" s="12" t="s">
+        <v>123</v>
+      </c>
+      <c r="E42" s="12" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="12"/>
+      <c r="B43" s="12"/>
+      <c r="C43" s="12" t="s">
+        <v>177</v>
+      </c>
+      <c r="D43" s="12" t="s">
+        <v>123</v>
+      </c>
+      <c r="E43" s="12" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="12"/>
+      <c r="B44" s="12"/>
+      <c r="C44" s="12" t="s">
+        <v>179</v>
+      </c>
+      <c r="D44" s="12" t="s">
+        <v>123</v>
+      </c>
+      <c r="E44" s="12"/>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="12"/>
+      <c r="B45" s="12"/>
+      <c r="C45" s="12" t="s">
+        <v>151</v>
+      </c>
+      <c r="D45" s="12" t="s">
+        <v>152</v>
+      </c>
+      <c r="E45" s="12"/>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="3" t="s">
+        <v>180</v>
+      </c>
+      <c r="B46" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="C46" s="11" t="s">
+        <v>139</v>
+      </c>
+      <c r="D46" s="11" t="s">
+        <v>140</v>
+      </c>
+      <c r="E46" s="11"/>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="12"/>
+      <c r="B47" s="12"/>
+      <c r="C47" s="12" t="s">
+        <v>119</v>
+      </c>
+      <c r="D47" s="12" t="s">
+        <v>123</v>
+      </c>
+      <c r="E47" s="12"/>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="7" t="s">
-        <v>87</v>
-      </c>
-      <c r="B48" s="7"/>
-      <c r="C48" s="7"/>
-      <c r="D48" s="8" t="n">
-        <f aca="false">D4+D9+D18+D31+D38+D42</f>
-        <v>56.5</v>
-      </c>
+      <c r="A48" s="12"/>
+      <c r="B48" s="12"/>
+      <c r="C48" s="12" t="s">
+        <v>154</v>
+      </c>
+      <c r="D48" s="12" t="s">
+        <v>123</v>
+      </c>
+      <c r="E48" s="12" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="12"/>
+      <c r="B49" s="12"/>
+      <c r="C49" s="12" t="s">
+        <v>156</v>
+      </c>
+      <c r="D49" s="12" t="s">
+        <v>123</v>
+      </c>
+      <c r="E49" s="12"/>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="9" t="s">
-        <v>88</v>
-      </c>
+      <c r="A50" s="12"/>
+      <c r="B50" s="12"/>
+      <c r="C50" s="12" t="s">
+        <v>182</v>
+      </c>
+      <c r="D50" s="12" t="s">
+        <v>123</v>
+      </c>
+      <c r="E50" s="12"/>
+    </row>
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A51" s="12"/>
+      <c r="B51" s="12"/>
+      <c r="C51" s="12" t="s">
+        <v>183</v>
+      </c>
+      <c r="D51" s="12" t="s">
+        <v>152</v>
+      </c>
+      <c r="E51" s="12" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A52" s="12"/>
+      <c r="B52" s="12"/>
+      <c r="C52" s="12" t="s">
+        <v>151</v>
+      </c>
+      <c r="D52" s="12" t="s">
+        <v>152</v>
+      </c>
+      <c r="E52" s="12"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>

<commit_message>
Fold setup and testing into each feature of the estimate
Each feature now carries its own setup and test-and-fix work; total is 60h.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016VxfYAmeTkhYFto1GdTc34
</commit_message>
<xml_diff>
--- a/Store_Shield_Estimation.xlsx
+++ b/Store_Shield_Estimation.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="291" uniqueCount="201">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="283" uniqueCount="192">
   <si>
     <t xml:space="preserve">Store Shield - Estimate</t>
   </si>
@@ -41,25 +41,97 @@
     <t xml:space="preserve">Hours</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Setup</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Create app</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Make the Shopify app and run it on the dev store</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NEW sessions (comes with Shopify template)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Shop settings</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Default settings saved on install</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NEW settings: shop, bot_checks (off/monitor/block each), blocked_asns, blocked_countries, speed_limit, alert_email</t>
+    <t xml:space="preserve">1. Bot Block</t>
+  </si>
+  <si>
+    <t xml:space="preserve">App &amp; settings</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Create the Shopify app, run it on the dev store, save default settings</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NEW sessions (Shopify template); NEW settings: shop, bot_checks (off/monitor/block each), blocked_asns, blocked_countries, speed_limit, alert_email</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Store script</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Small script on every store page</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Automation check</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Spot Puppeteer, Selenium, Playwright, headless</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Extension &amp; injection scan</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Spot scraper/scalper extensions in the page</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Visitor check API</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Receive results, get real IP, decide block or not</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NEW visits: shop, device_id, ip, asn, country, page, flags, action, created_at</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Data-centre / VPN / Tor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IP lookup with GeoLite2, cloud IP lists, Tor list</t>
+  </si>
+  <si>
+    <t xml:space="preserve">- (lists kept as files, refreshed daily)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ASN &amp; country block</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Block networks or countries the merchant picks</t>
+  </si>
+  <si>
+    <t xml:space="preserve">- (reads settings)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Speed limit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Too many pages from one IP or subnet</t>
+  </si>
+  <si>
+    <t xml:space="preserve">- (counter kept in memory)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Good-bot allowlist</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Never block real Google, Bing, Facebook bots</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Block screen &amp; monitor mode</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Block page with contact link; pass result to checkout</t>
+  </si>
+  <si>
+    <t xml:space="preserve">- (result saved on the Shopify cart)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Test &amp; fix</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Run fake bots (plain, stealth, data-centre IP) and fix issues</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2. Rules Engine</t>
   </si>
   <si>
     <t xml:space="preserve">Test store</t>
@@ -68,7 +140,88 @@
     <t xml:space="preserve">Sample products, COD and a test card gateway</t>
   </si>
   <si>
-    <t xml:space="preserve">-</t>
+    <t xml:space="preserve">Rule engine core</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Store rules, check conditions with ALL/ANY, Live/Test/Off</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NEW rules: shop, name, stage, match, conditions, actions, status, priority, times_triggered, last_triggered_at</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hide payment methods</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hide COD or other methods at checkout (Shopify Function)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">- (checkout rules copied to a Shopify metafield)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">New order trigger</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Get full order details when an order is placed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NEW order_checks: shop, order_id, order_name, ip, email_hash, phone_hash, total, matched_rules, actions_taken, status, created_at</t>
+  </si>
+  <si>
+    <t xml:space="preserve">After-order conditions</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Address mismatch, IP country, Shopify risk, disposable email, cart value...</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Velocity condition</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Many orders from same IP / email / phone in X hours</t>
+  </si>
+  <si>
+    <t xml:space="preserve">- (reads order_checks)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fraud history condition</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Matches a past fraud email, phone or address</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NEW fraud_list: shop, type, value_hash, order_id, created_at</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Action: Put in review</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pause fulfilment and list it for review</t>
+  </si>
+  <si>
+    <t xml:space="preserve">- (updates order_checks.status)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Action: Auto-cancel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cancel with refund / restock / email options</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Action: Tag</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Add tags to the order and/or customer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Action: Email alert (optional)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Email the merchant when a rule fires</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rule conflicts</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cancel beats review; all tags applied</t>
   </si>
   <si>
     <t xml:space="preserve">Privacy webhooks</t>
@@ -80,166 +233,10 @@
     <t xml:space="preserve">- (deletes rows for a customer or shop)</t>
   </si>
   <si>
-    <t xml:space="preserve">2. Bot Block</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Store script</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Small script on every store page</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Automation check</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Spot Puppeteer, Selenium, Playwright, headless</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Extension &amp; injection scan</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Spot scraper/scalper extensions in the page</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Visitor check API</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Receive results, get real IP, decide block or not</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NEW visits: shop, device_id, ip, asn, country, page, flags, action, created_at</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Data-centre / VPN / Tor</t>
-  </si>
-  <si>
-    <t xml:space="preserve">IP lookup with GeoLite2, cloud IP lists, Tor list</t>
-  </si>
-  <si>
-    <t xml:space="preserve">- (lists kept as files, refreshed daily)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ASN &amp; country block</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Block networks or countries the merchant picks</t>
-  </si>
-  <si>
-    <t xml:space="preserve">- (reads settings)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Speed limit</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Too many pages from one IP or subnet</t>
-  </si>
-  <si>
-    <t xml:space="preserve">- (counter kept in memory)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Good-bot allowlist</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Never block real Google, Bing, Facebook bots</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Block screen &amp; monitor mode</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Block page with contact link; pass result to checkout</t>
-  </si>
-  <si>
-    <t xml:space="preserve">- (result saved on the Shopify cart)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3. Rules Engine</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Rule engine core</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Store rules, check conditions with ALL/ANY, Live/Test/Off</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NEW rules: shop, name, stage, match, conditions, actions, status, priority, times_triggered, last_triggered_at</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hide payment methods</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hide COD or other methods at checkout (Shopify Function)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">- (checkout rules copied to a Shopify metafield)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">New order trigger</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Get full order details when an order is placed</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NEW order_checks: shop, order_id, order_name, ip, email_hash, phone_hash, total, matched_rules, actions_taken, status, created_at</t>
-  </si>
-  <si>
-    <t xml:space="preserve">After-order conditions</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Address mismatch, IP country, Shopify risk, disposable email, cart value...</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Velocity condition</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Many orders from same IP / email / phone in X hours</t>
-  </si>
-  <si>
-    <t xml:space="preserve">- (reads order_checks)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fraud history condition</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Matches a past fraud email, phone or address</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NEW fraud_list: shop, type, value_hash, order_id, created_at</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Action: Put in review</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pause fulfilment and list it for review</t>
-  </si>
-  <si>
-    <t xml:space="preserve">- (updates order_checks.status)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Action: Auto-cancel</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cancel with refund / restock / email options</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Action: Tag</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Add tags to the order and/or customer</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Action: Email alert (optional)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Email the merchant when a rule fires</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Rule conflicts</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cancel beats review; all tags applied</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4. Pages</t>
+    <t xml:space="preserve">Unit tests, one test order per action, check COD really hides, fix issues</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3. Admin Pages</t>
   </si>
   <si>
     <t xml:space="preserve">Menu &amp; layout</t>
@@ -314,27 +311,6 @@
     <t xml:space="preserve">Top reasons, top rules, trend over time</t>
   </si>
   <si>
-    <t xml:space="preserve">5. Testing &amp; Launch</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bot tests</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fake bots (plain, stealth, data-centre IP) against the store</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Rule tests</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Unit tests + one test order per action</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Checkout test</t>
-  </si>
-  <si>
-    <t xml:space="preserve">COD really disappears for matching carts</t>
-  </si>
-  <si>
     <t xml:space="preserve">Go live</t>
   </si>
   <si>
@@ -344,10 +320,7 @@
     <t xml:space="preserve">Move from SQLite to Postgres</t>
   </si>
   <si>
-    <t xml:space="preserve">Fix bugs</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Spare time for problems</t>
+    <t xml:space="preserve">Run the full story end to end on the live app, fix issues</t>
   </si>
   <si>
     <t xml:space="preserve">TOTAL</t>
@@ -1078,7 +1051,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E55"/>
+  <dimension ref="A1:E51"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="20"/>
@@ -1118,11 +1091,11 @@
       <c r="C4" s="3"/>
       <c r="D4" s="3"/>
       <c r="E4" s="4" t="n">
-        <f aca="false">SUM(E5:E8)</f>
-        <v>4.5</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <f aca="false">SUM(E5:E15)</f>
+        <v>18</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="5"/>
       <c r="B5" s="5" t="s">
         <v>7</v>
@@ -1134,10 +1107,10 @@
         <v>9</v>
       </c>
       <c r="E5" s="6" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>2.5</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="5"/>
       <c r="B6" s="5" t="s">
         <v>10</v>
@@ -1149,7 +1122,7 @@
         <v>12</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>0.5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1161,37 +1134,40 @@
         <v>14</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="E7" s="6" t="n">
-        <v>1</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="5"/>
       <c r="B8" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C8" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="C8" s="5" t="s">
+      <c r="D8" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="E8" s="6" t="n">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="5"/>
+      <c r="B9" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="D8" s="5" t="s">
+      <c r="C9" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="E8" s="6" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="3" t="s">
+      <c r="D9" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="B9" s="3"/>
-      <c r="C9" s="3"/>
-      <c r="D9" s="3"/>
-      <c r="E9" s="4" t="n">
-        <f aca="false">SUM(E10:E18)</f>
-        <v>13</v>
+      <c r="E9" s="6" t="n">
+        <v>1.5</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1203,112 +1179,109 @@
         <v>21</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="E10" s="6" t="n">
-        <v>2</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="5"/>
       <c r="B11" s="5" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="E11" s="6" t="n">
-        <v>1.5</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="5"/>
       <c r="B12" s="5" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>15</v>
+        <v>28</v>
       </c>
       <c r="E12" s="6" t="n">
-        <v>1.5</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="5"/>
       <c r="B13" s="5" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>28</v>
+        <v>12</v>
       </c>
       <c r="E13" s="6" t="n">
-        <v>1.5</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="5"/>
       <c r="B14" s="5" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="E14" s="6" t="n">
-        <v>2.5</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="5"/>
       <c r="B15" s="5" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>34</v>
+        <v>12</v>
       </c>
       <c r="E15" s="6" t="n">
-        <v>0.5</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="5"/>
-      <c r="B16" s="5" t="s">
-        <v>35</v>
-      </c>
-      <c r="C16" s="5" t="s">
+      <c r="A16" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="D16" s="5" t="s">
-        <v>37</v>
-      </c>
-      <c r="E16" s="6" t="n">
-        <v>1</v>
+      <c r="B16" s="3"/>
+      <c r="C16" s="3"/>
+      <c r="D16" s="3"/>
+      <c r="E16" s="4" t="n">
+        <f aca="false">SUM(E17:E30)</f>
+        <v>23</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="5"/>
       <c r="B17" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="C17" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="C17" s="5" t="s">
-        <v>39</v>
-      </c>
       <c r="D17" s="5" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="E17" s="6" t="n">
         <v>1</v>
@@ -1317,61 +1290,64 @@
     <row r="18" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="5"/>
       <c r="B18" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="C18" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="C18" s="5" t="s">
+      <c r="D18" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="D18" s="5" t="s">
+      <c r="E18" s="6" t="n">
+        <v>2.5</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="5"/>
+      <c r="B19" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="E18" s="6" t="n">
-        <v>1.5</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="3" t="s">
+      <c r="C19" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="B19" s="3"/>
-      <c r="C19" s="3"/>
-      <c r="D19" s="3"/>
-      <c r="E19" s="4" t="n">
-        <f aca="false">SUM(E20:E30)</f>
-        <v>17</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D19" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="E19" s="6" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="5"/>
       <c r="B20" s="5" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="D20" s="5" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="E20" s="6" t="n">
-        <v>2.5</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="5"/>
       <c r="B21" s="5" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D21" s="5" t="s">
-        <v>49</v>
+        <v>12</v>
       </c>
       <c r="E21" s="6" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="5"/>
       <c r="B22" s="5" t="s">
         <v>50</v>
@@ -1383,10 +1359,10 @@
         <v>52</v>
       </c>
       <c r="E22" s="6" t="n">
-        <v>1.5</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="5"/>
       <c r="B23" s="5" t="s">
         <v>53</v>
@@ -1395,37 +1371,37 @@
         <v>54</v>
       </c>
       <c r="D23" s="5" t="s">
-        <v>15</v>
+        <v>55</v>
       </c>
       <c r="E23" s="6" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="5"/>
       <c r="B24" s="5" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D24" s="5" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="E24" s="6" t="n">
-        <v>1</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="5"/>
       <c r="B25" s="5" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D25" s="5" t="s">
-        <v>60</v>
+        <v>12</v>
       </c>
       <c r="E25" s="6" t="n">
         <v>1.5</v>
@@ -1440,37 +1416,37 @@
         <v>62</v>
       </c>
       <c r="D26" s="5" t="s">
-        <v>63</v>
+        <v>12</v>
       </c>
       <c r="E26" s="6" t="n">
-        <v>1.5</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="5"/>
-      <c r="B27" s="5" t="s">
+      <c r="B27" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="C27" s="5" t="s">
         <v>64</v>
       </c>
-      <c r="C27" s="5" t="s">
-        <v>65</v>
-      </c>
       <c r="D27" s="5" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="E27" s="6" t="n">
-        <v>1.5</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="5"/>
       <c r="B28" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="C28" s="5" t="s">
         <v>66</v>
       </c>
-      <c r="C28" s="5" t="s">
-        <v>67</v>
-      </c>
       <c r="D28" s="5" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="E28" s="6" t="n">
         <v>0.5</v>
@@ -1478,56 +1454,56 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="5"/>
-      <c r="B29" s="7" t="s">
+      <c r="B29" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="C29" s="5" t="s">
         <v>68</v>
       </c>
-      <c r="C29" s="5" t="s">
+      <c r="D29" s="5" t="s">
         <v>69</v>
       </c>
-      <c r="D29" s="5" t="s">
-        <v>15</v>
-      </c>
       <c r="E29" s="6" t="n">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="5"/>
       <c r="B30" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="C30" s="5" t="s">
         <v>70</v>
       </c>
-      <c r="C30" s="5" t="s">
-        <v>71</v>
-      </c>
       <c r="D30" s="5" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="E30" s="6" t="n">
-        <v>0.5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="3" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B31" s="3"/>
       <c r="C31" s="3"/>
       <c r="D31" s="3"/>
       <c r="E31" s="4" t="n">
-        <f aca="false">SUM(E32:E41)</f>
-        <v>14.5</v>
+        <f aca="false">SUM(E32:E43)</f>
+        <v>19</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="5"/>
       <c r="B32" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="C32" s="5" t="s">
         <v>73</v>
       </c>
-      <c r="C32" s="5" t="s">
-        <v>74</v>
-      </c>
       <c r="D32" s="5" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="E32" s="6" t="n">
         <v>0.5</v>
@@ -1536,13 +1512,13 @@
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="5"/>
       <c r="B33" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="C33" s="5" t="s">
         <v>75</v>
       </c>
-      <c r="C33" s="5" t="s">
-        <v>76</v>
-      </c>
       <c r="D33" s="5" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="E33" s="6" t="n">
         <v>1.5</v>
@@ -1551,13 +1527,13 @@
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="5"/>
       <c r="B34" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="C34" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="C34" s="5" t="s">
-        <v>78</v>
-      </c>
       <c r="D34" s="5" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="E34" s="6" t="n">
         <v>3.5</v>
@@ -1566,13 +1542,13 @@
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="5"/>
       <c r="B35" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="C35" s="5" t="s">
         <v>79</v>
       </c>
-      <c r="C35" s="5" t="s">
-        <v>80</v>
-      </c>
       <c r="D35" s="5" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="E35" s="6" t="n">
         <v>1</v>
@@ -1581,13 +1557,13 @@
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="5"/>
       <c r="B36" s="5" t="s">
+        <v>80</v>
+      </c>
+      <c r="C36" s="5" t="s">
         <v>81</v>
       </c>
-      <c r="C36" s="5" t="s">
-        <v>82</v>
-      </c>
       <c r="D36" s="5" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="E36" s="6" t="n">
         <v>1.5</v>
@@ -1596,13 +1572,13 @@
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="5"/>
       <c r="B37" s="5" t="s">
+        <v>82</v>
+      </c>
+      <c r="C37" s="5" t="s">
         <v>83</v>
       </c>
-      <c r="C37" s="5" t="s">
+      <c r="D37" s="5" t="s">
         <v>84</v>
-      </c>
-      <c r="D37" s="5" t="s">
-        <v>85</v>
       </c>
       <c r="E37" s="6" t="n">
         <v>2</v>
@@ -1611,13 +1587,13 @@
     <row r="38" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="5"/>
       <c r="B38" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="C38" s="5" t="s">
         <v>86</v>
       </c>
-      <c r="C38" s="5" t="s">
+      <c r="D38" s="5" t="s">
         <v>87</v>
-      </c>
-      <c r="D38" s="5" t="s">
-        <v>88</v>
       </c>
       <c r="E38" s="6" t="n">
         <v>1.5</v>
@@ -1626,13 +1602,13 @@
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="5"/>
       <c r="B39" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="C39" s="5" t="s">
         <v>89</v>
       </c>
-      <c r="C39" s="5" t="s">
+      <c r="D39" s="5" t="s">
         <v>90</v>
-      </c>
-      <c r="D39" s="5" t="s">
-        <v>91</v>
       </c>
       <c r="E39" s="6" t="n">
         <v>1</v>
@@ -1641,13 +1617,13 @@
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="5"/>
       <c r="B40" s="5" t="s">
+        <v>91</v>
+      </c>
+      <c r="C40" s="5" t="s">
         <v>92</v>
       </c>
-      <c r="C40" s="5" t="s">
+      <c r="D40" s="5" t="s">
         <v>93</v>
-      </c>
-      <c r="D40" s="5" t="s">
-        <v>94</v>
       </c>
       <c r="E40" s="6" t="n">
         <v>1</v>
@@ -1656,159 +1632,102 @@
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="5"/>
       <c r="B41" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="C41" s="5" t="s">
         <v>95</v>
       </c>
-      <c r="C41" s="5" t="s">
-        <v>96</v>
-      </c>
       <c r="D41" s="5" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="E41" s="6" t="n">
         <v>1</v>
       </c>
     </row>
-    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="3" t="s">
+    <row r="42" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="5"/>
+      <c r="B42" s="5" t="s">
+        <v>96</v>
+      </c>
+      <c r="C42" s="5" t="s">
         <v>97</v>
       </c>
-      <c r="B42" s="3"/>
-      <c r="C42" s="3"/>
-      <c r="D42" s="3"/>
-      <c r="E42" s="4" t="n">
-        <f aca="false">SUM(E43:E47)</f>
-        <v>9.5</v>
+      <c r="D42" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="E42" s="6" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="5"/>
       <c r="B43" s="5" t="s">
-        <v>98</v>
+        <v>34</v>
       </c>
       <c r="C43" s="5" t="s">
         <v>99</v>
       </c>
       <c r="D43" s="5" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="E43" s="6" t="n">
-        <v>1.5</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="5"/>
-      <c r="B44" s="5" t="s">
+      <c r="A44" s="8" t="s">
         <v>100</v>
       </c>
-      <c r="C44" s="5" t="s">
+      <c r="B44" s="8"/>
+      <c r="C44" s="8"/>
+      <c r="D44" s="8"/>
+      <c r="E44" s="9" t="n">
+        <f aca="false">E4+E16+E31</f>
+        <v>60</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="8" t="s">
         <v>101</v>
       </c>
-      <c r="D44" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="E44" s="6" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="5"/>
-      <c r="B45" s="5" t="s">
+      <c r="B45" s="8"/>
+      <c r="C45" s="8"/>
+      <c r="D45" s="8"/>
+      <c r="E45" s="9" t="n">
+        <f aca="false">E27+E35+E41</f>
+        <v>2.5</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="8" t="s">
         <v>102</v>
       </c>
-      <c r="C45" s="5" t="s">
+      <c r="B46" s="8"/>
+      <c r="C46" s="8"/>
+      <c r="D46" s="8"/>
+      <c r="E46" s="9" t="n">
+        <f aca="false">E44-E45</f>
+        <v>57.5</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="10" t="s">
         <v>103</v>
       </c>
-      <c r="D45" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="E45" s="6" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="46" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="5"/>
-      <c r="B46" s="5" t="s">
+    </row>
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="10" t="s">
         <v>104</v>
       </c>
-      <c r="C46" s="5" t="s">
+    </row>
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="10" t="s">
         <v>105</v>
       </c>
-      <c r="D46" s="5" t="s">
+    </row>
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A51" s="10" t="s">
         <v>106</v>
-      </c>
-      <c r="E46" s="6" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="5"/>
-      <c r="B47" s="5" t="s">
-        <v>107</v>
-      </c>
-      <c r="C47" s="5" t="s">
-        <v>108</v>
-      </c>
-      <c r="D47" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="E47" s="6" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="8" t="s">
-        <v>109</v>
-      </c>
-      <c r="B48" s="8"/>
-      <c r="C48" s="8"/>
-      <c r="D48" s="8"/>
-      <c r="E48" s="9" t="n">
-        <f aca="false">E4+E9+E19+E31+E42</f>
-        <v>58.5</v>
-      </c>
-    </row>
-    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="8" t="s">
-        <v>110</v>
-      </c>
-      <c r="B49" s="8"/>
-      <c r="C49" s="8"/>
-      <c r="D49" s="8"/>
-      <c r="E49" s="9" t="n">
-        <f aca="false">E29+E35+E41</f>
-        <v>2.5</v>
-      </c>
-    </row>
-    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="8" t="s">
-        <v>111</v>
-      </c>
-      <c r="B50" s="8"/>
-      <c r="C50" s="8"/>
-      <c r="D50" s="8"/>
-      <c r="E50" s="9" t="n">
-        <f aca="false">E48-E49</f>
-        <v>56</v>
-      </c>
-    </row>
-    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="10" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A53" s="10" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A54" s="10" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A55" s="10" t="s">
-        <v>115</v>
       </c>
     </row>
   </sheetData>
@@ -1839,135 +1758,135 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>116</v>
+        <v>107</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="11" t="s">
-        <v>117</v>
+        <v>108</v>
       </c>
       <c r="B3" s="11" t="s">
-        <v>118</v>
+        <v>109</v>
       </c>
       <c r="C3" s="11" t="s">
-        <v>119</v>
+        <v>110</v>
       </c>
       <c r="D3" s="11" t="s">
-        <v>120</v>
+        <v>111</v>
       </c>
       <c r="E3" s="11" t="s">
-        <v>121</v>
+        <v>112</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>122</v>
+        <v>113</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>7</v>
       </c>
       <c r="C4" s="12" t="s">
-        <v>123</v>
+        <v>114</v>
       </c>
       <c r="D4" s="12"/>
       <c r="E4" s="12" t="s">
-        <v>124</v>
+        <v>115</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>125</v>
+        <v>116</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="C5" s="12" t="s">
-        <v>126</v>
+        <v>117</v>
       </c>
       <c r="D5" s="12" t="s">
-        <v>127</v>
+        <v>118</v>
       </c>
       <c r="E5" s="12" t="s">
-        <v>128</v>
+        <v>119</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="13"/>
       <c r="B6" s="13"/>
       <c r="C6" s="13" t="s">
-        <v>129</v>
+        <v>120</v>
       </c>
       <c r="D6" s="13" t="s">
-        <v>130</v>
+        <v>121</v>
       </c>
       <c r="E6" s="13" t="s">
-        <v>131</v>
+        <v>122</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="13"/>
       <c r="B7" s="13"/>
       <c r="C7" s="13" t="s">
-        <v>132</v>
+        <v>123</v>
       </c>
       <c r="D7" s="13" t="s">
-        <v>130</v>
+        <v>121</v>
       </c>
       <c r="E7" s="13" t="s">
-        <v>133</v>
+        <v>124</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="13"/>
       <c r="B8" s="13"/>
       <c r="C8" s="13" t="s">
-        <v>134</v>
+        <v>125</v>
       </c>
       <c r="D8" s="13" t="s">
-        <v>130</v>
+        <v>121</v>
       </c>
       <c r="E8" s="13" t="s">
-        <v>135</v>
+        <v>126</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="13"/>
       <c r="B9" s="13"/>
       <c r="C9" s="13" t="s">
-        <v>136</v>
+        <v>127</v>
       </c>
       <c r="D9" s="13" t="s">
-        <v>137</v>
+        <v>128</v>
       </c>
       <c r="E9" s="13" t="s">
-        <v>138</v>
+        <v>129</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="13"/>
       <c r="B10" s="13"/>
       <c r="C10" s="13" t="s">
-        <v>139</v>
+        <v>130</v>
       </c>
       <c r="D10" s="13" t="s">
-        <v>140</v>
+        <v>131</v>
       </c>
       <c r="E10" s="13" t="s">
-        <v>141</v>
+        <v>132</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>142</v>
+        <v>133</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>26</v>
+        <v>17</v>
       </c>
       <c r="C11" s="12" t="s">
-        <v>143</v>
+        <v>134</v>
       </c>
       <c r="D11" s="12" t="s">
-        <v>144</v>
+        <v>135</v>
       </c>
       <c r="E11" s="12"/>
     </row>
@@ -1975,10 +1894,10 @@
       <c r="A12" s="13"/>
       <c r="B12" s="13"/>
       <c r="C12" s="13" t="s">
-        <v>126</v>
+        <v>117</v>
       </c>
       <c r="D12" s="13" t="s">
-        <v>140</v>
+        <v>131</v>
       </c>
       <c r="E12" s="13"/>
     </row>
@@ -1986,36 +1905,36 @@
       <c r="A13" s="13"/>
       <c r="B13" s="13"/>
       <c r="C13" s="13" t="s">
-        <v>145</v>
+        <v>136</v>
       </c>
       <c r="D13" s="13" t="s">
-        <v>140</v>
+        <v>131</v>
       </c>
       <c r="E13" s="13" t="s">
-        <v>146</v>
+        <v>137</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="13"/>
       <c r="B14" s="13"/>
       <c r="C14" s="13" t="s">
-        <v>147</v>
+        <v>138</v>
       </c>
       <c r="D14" s="13" t="s">
-        <v>140</v>
+        <v>131</v>
       </c>
       <c r="E14" s="13" t="s">
-        <v>148</v>
+        <v>139</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="13"/>
       <c r="B15" s="13"/>
       <c r="C15" s="13" t="s">
-        <v>149</v>
+        <v>140</v>
       </c>
       <c r="D15" s="13" t="s">
-        <v>140</v>
+        <v>131</v>
       </c>
       <c r="E15" s="13"/>
     </row>
@@ -2023,53 +1942,53 @@
       <c r="A16" s="13"/>
       <c r="B16" s="13"/>
       <c r="C16" s="13" t="s">
-        <v>150</v>
+        <v>141</v>
       </c>
       <c r="D16" s="13" t="s">
-        <v>130</v>
+        <v>121</v>
       </c>
       <c r="E16" s="13" t="s">
-        <v>151</v>
+        <v>142</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="13"/>
       <c r="B17" s="13"/>
       <c r="C17" s="13" t="s">
-        <v>152</v>
+        <v>143</v>
       </c>
       <c r="D17" s="13" t="s">
-        <v>140</v>
+        <v>131</v>
       </c>
       <c r="E17" s="13" t="s">
-        <v>153</v>
+        <v>144</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="13"/>
       <c r="B18" s="13"/>
       <c r="C18" s="13" t="s">
-        <v>154</v>
+        <v>145</v>
       </c>
       <c r="D18" s="13" t="s">
-        <v>155</v>
+        <v>146</v>
       </c>
       <c r="E18" s="13" t="s">
-        <v>156</v>
+        <v>147</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="3" t="s">
-        <v>157</v>
+        <v>148</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="C19" s="12" t="s">
-        <v>143</v>
+        <v>134</v>
       </c>
       <c r="D19" s="12" t="s">
-        <v>144</v>
+        <v>135</v>
       </c>
       <c r="E19" s="12"/>
     </row>
@@ -2077,10 +1996,10 @@
       <c r="A20" s="13"/>
       <c r="B20" s="13"/>
       <c r="C20" s="13" t="s">
-        <v>126</v>
+        <v>117</v>
       </c>
       <c r="D20" s="13" t="s">
-        <v>140</v>
+        <v>131</v>
       </c>
       <c r="E20" s="13"/>
     </row>
@@ -2088,10 +2007,10 @@
       <c r="A21" s="13"/>
       <c r="B21" s="13"/>
       <c r="C21" s="13" t="s">
-        <v>158</v>
+        <v>149</v>
       </c>
       <c r="D21" s="13" t="s">
-        <v>140</v>
+        <v>131</v>
       </c>
       <c r="E21" s="13"/>
     </row>
@@ -2099,75 +2018,75 @@
       <c r="A22" s="13"/>
       <c r="B22" s="13"/>
       <c r="C22" s="13" t="s">
-        <v>159</v>
+        <v>150</v>
       </c>
       <c r="D22" s="13" t="s">
-        <v>140</v>
+        <v>131</v>
       </c>
       <c r="E22" s="13" t="s">
-        <v>160</v>
+        <v>151</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="13"/>
       <c r="B23" s="13"/>
       <c r="C23" s="13" t="s">
-        <v>161</v>
+        <v>152</v>
       </c>
       <c r="D23" s="13" t="s">
-        <v>140</v>
+        <v>131</v>
       </c>
       <c r="E23" s="13" t="s">
-        <v>162</v>
+        <v>153</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="13"/>
       <c r="B24" s="13"/>
       <c r="C24" s="13" t="s">
-        <v>163</v>
+        <v>154</v>
       </c>
       <c r="D24" s="13" t="s">
-        <v>130</v>
+        <v>121</v>
       </c>
       <c r="E24" s="13" t="s">
-        <v>164</v>
+        <v>155</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="13"/>
       <c r="B25" s="13"/>
       <c r="C25" s="13" t="s">
-        <v>165</v>
+        <v>156</v>
       </c>
       <c r="D25" s="13" t="s">
-        <v>130</v>
+        <v>121</v>
       </c>
       <c r="E25" s="13" t="s">
-        <v>166</v>
+        <v>157</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="13"/>
       <c r="B26" s="13"/>
       <c r="C26" s="13" t="s">
-        <v>167</v>
+        <v>158</v>
       </c>
       <c r="D26" s="13" t="s">
-        <v>140</v>
+        <v>131</v>
       </c>
       <c r="E26" s="13" t="s">
-        <v>168</v>
+        <v>159</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="13"/>
       <c r="B27" s="13"/>
       <c r="C27" s="13" t="s">
-        <v>169</v>
+        <v>160</v>
       </c>
       <c r="D27" s="13" t="s">
-        <v>137</v>
+        <v>128</v>
       </c>
       <c r="E27" s="13"/>
     </row>
@@ -2175,27 +2094,27 @@
       <c r="A28" s="13"/>
       <c r="B28" s="13"/>
       <c r="C28" s="13" t="s">
-        <v>170</v>
+        <v>161</v>
       </c>
       <c r="D28" s="13" t="s">
-        <v>171</v>
+        <v>162</v>
       </c>
       <c r="E28" s="13" t="s">
-        <v>172</v>
+        <v>163</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="3" t="s">
-        <v>173</v>
+        <v>164</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="C29" s="12" t="s">
-        <v>143</v>
+        <v>134</v>
       </c>
       <c r="D29" s="12" t="s">
-        <v>144</v>
+        <v>135</v>
       </c>
       <c r="E29" s="12"/>
     </row>
@@ -2203,10 +2122,10 @@
       <c r="A30" s="13"/>
       <c r="B30" s="13"/>
       <c r="C30" s="13" t="s">
-        <v>126</v>
+        <v>117</v>
       </c>
       <c r="D30" s="13" t="s">
-        <v>140</v>
+        <v>131</v>
       </c>
       <c r="E30" s="13"/>
     </row>
@@ -2214,49 +2133,49 @@
       <c r="A31" s="13"/>
       <c r="B31" s="13"/>
       <c r="C31" s="13" t="s">
-        <v>174</v>
+        <v>165</v>
       </c>
       <c r="D31" s="13" t="s">
-        <v>140</v>
+        <v>131</v>
       </c>
       <c r="E31" s="13" t="s">
-        <v>175</v>
+        <v>166</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="13"/>
       <c r="B32" s="13"/>
       <c r="C32" s="13" t="s">
-        <v>176</v>
+        <v>167</v>
       </c>
       <c r="D32" s="13" t="s">
-        <v>140</v>
+        <v>131</v>
       </c>
       <c r="E32" s="13" t="s">
-        <v>177</v>
+        <v>168</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="13"/>
       <c r="B33" s="13"/>
       <c r="C33" s="13" t="s">
-        <v>178</v>
+        <v>169</v>
       </c>
       <c r="D33" s="13" t="s">
-        <v>140</v>
+        <v>131</v>
       </c>
       <c r="E33" s="13" t="s">
-        <v>179</v>
+        <v>170</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="13"/>
       <c r="B34" s="13"/>
       <c r="C34" s="13" t="s">
-        <v>180</v>
+        <v>171</v>
       </c>
       <c r="D34" s="13" t="s">
-        <v>181</v>
+        <v>172</v>
       </c>
       <c r="E34" s="13"/>
     </row>
@@ -2264,23 +2183,23 @@
       <c r="A35" s="13"/>
       <c r="B35" s="13"/>
       <c r="C35" s="13" t="s">
-        <v>182</v>
+        <v>173</v>
       </c>
       <c r="D35" s="13" t="s">
-        <v>130</v>
+        <v>121</v>
       </c>
       <c r="E35" s="13" t="s">
-        <v>183</v>
+        <v>174</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="13"/>
       <c r="B36" s="13"/>
       <c r="C36" s="13" t="s">
-        <v>184</v>
+        <v>175</v>
       </c>
       <c r="D36" s="13" t="s">
-        <v>130</v>
+        <v>121</v>
       </c>
       <c r="E36" s="13"/>
     </row>
@@ -2288,40 +2207,40 @@
       <c r="A37" s="13"/>
       <c r="B37" s="13"/>
       <c r="C37" s="13" t="s">
-        <v>167</v>
+        <v>158</v>
       </c>
       <c r="D37" s="13" t="s">
-        <v>140</v>
+        <v>131</v>
       </c>
       <c r="E37" s="13" t="s">
-        <v>185</v>
+        <v>176</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="13"/>
       <c r="B38" s="13"/>
       <c r="C38" s="13" t="s">
-        <v>154</v>
+        <v>145</v>
       </c>
       <c r="D38" s="13" t="s">
-        <v>155</v>
+        <v>146</v>
       </c>
       <c r="E38" s="13" t="s">
-        <v>186</v>
+        <v>177</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="3" t="s">
-        <v>187</v>
+        <v>178</v>
       </c>
       <c r="B39" s="3" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="C39" s="12" t="s">
-        <v>143</v>
+        <v>134</v>
       </c>
       <c r="D39" s="12" t="s">
-        <v>144</v>
+        <v>135</v>
       </c>
       <c r="E39" s="12"/>
     </row>
@@ -2329,10 +2248,10 @@
       <c r="A40" s="13"/>
       <c r="B40" s="13"/>
       <c r="C40" s="13" t="s">
-        <v>126</v>
+        <v>117</v>
       </c>
       <c r="D40" s="13" t="s">
-        <v>140</v>
+        <v>131</v>
       </c>
       <c r="E40" s="13"/>
     </row>
@@ -2340,64 +2259,64 @@
       <c r="A41" s="13"/>
       <c r="B41" s="13"/>
       <c r="C41" s="13" t="s">
-        <v>188</v>
+        <v>179</v>
       </c>
       <c r="D41" s="13" t="s">
-        <v>140</v>
+        <v>131</v>
       </c>
       <c r="E41" s="13" t="s">
-        <v>189</v>
+        <v>180</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="13"/>
       <c r="B42" s="13"/>
       <c r="C42" s="13" t="s">
-        <v>190</v>
+        <v>181</v>
       </c>
       <c r="D42" s="13" t="s">
-        <v>140</v>
+        <v>131</v>
       </c>
       <c r="E42" s="13" t="s">
-        <v>191</v>
+        <v>182</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="13"/>
       <c r="B43" s="13"/>
       <c r="C43" s="13" t="s">
-        <v>192</v>
+        <v>183</v>
       </c>
       <c r="D43" s="13" t="s">
-        <v>140</v>
+        <v>131</v>
       </c>
       <c r="E43" s="13" t="s">
-        <v>193</v>
+        <v>184</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="13"/>
       <c r="B44" s="13"/>
       <c r="C44" s="13" t="s">
-        <v>154</v>
+        <v>145</v>
       </c>
       <c r="D44" s="13" t="s">
-        <v>155</v>
+        <v>146</v>
       </c>
       <c r="E44" s="13"/>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="3" t="s">
-        <v>194</v>
+        <v>185</v>
       </c>
       <c r="B45" s="3" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C45" s="12" t="s">
-        <v>143</v>
+        <v>134</v>
       </c>
       <c r="D45" s="12" t="s">
-        <v>144</v>
+        <v>135</v>
       </c>
       <c r="E45" s="12"/>
     </row>
@@ -2405,10 +2324,10 @@
       <c r="A46" s="13"/>
       <c r="B46" s="13"/>
       <c r="C46" s="13" t="s">
-        <v>126</v>
+        <v>117</v>
       </c>
       <c r="D46" s="13" t="s">
-        <v>140</v>
+        <v>131</v>
       </c>
       <c r="E46" s="13"/>
     </row>
@@ -2416,10 +2335,10 @@
       <c r="A47" s="13"/>
       <c r="B47" s="13"/>
       <c r="C47" s="13" t="s">
-        <v>192</v>
+        <v>183</v>
       </c>
       <c r="D47" s="13" t="s">
-        <v>140</v>
+        <v>131</v>
       </c>
       <c r="E47" s="13"/>
     </row>
@@ -2427,23 +2346,23 @@
       <c r="A48" s="13"/>
       <c r="B48" s="13"/>
       <c r="C48" s="13" t="s">
-        <v>152</v>
+        <v>143</v>
       </c>
       <c r="D48" s="13" t="s">
-        <v>140</v>
+        <v>131</v>
       </c>
       <c r="E48" s="13" t="s">
-        <v>195</v>
+        <v>186</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="13"/>
       <c r="B49" s="13"/>
       <c r="C49" s="13" t="s">
-        <v>196</v>
+        <v>187</v>
       </c>
       <c r="D49" s="13" t="s">
-        <v>140</v>
+        <v>131</v>
       </c>
       <c r="E49" s="13"/>
     </row>
@@ -2451,25 +2370,25 @@
       <c r="A50" s="13"/>
       <c r="B50" s="13"/>
       <c r="C50" s="13" t="s">
-        <v>154</v>
+        <v>145</v>
       </c>
       <c r="D50" s="13" t="s">
-        <v>155</v>
+        <v>146</v>
       </c>
       <c r="E50" s="13"/>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="3" t="s">
-        <v>197</v>
+        <v>188</v>
       </c>
       <c r="B51" s="3" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C51" s="12" t="s">
-        <v>143</v>
+        <v>134</v>
       </c>
       <c r="D51" s="12" t="s">
-        <v>144</v>
+        <v>135</v>
       </c>
       <c r="E51" s="12"/>
     </row>
@@ -2477,10 +2396,10 @@
       <c r="A52" s="13"/>
       <c r="B52" s="13"/>
       <c r="C52" s="13" t="s">
-        <v>126</v>
+        <v>117</v>
       </c>
       <c r="D52" s="13" t="s">
-        <v>140</v>
+        <v>131</v>
       </c>
       <c r="E52" s="13"/>
     </row>
@@ -2488,23 +2407,23 @@
       <c r="A53" s="13"/>
       <c r="B53" s="13"/>
       <c r="C53" s="13" t="s">
-        <v>188</v>
+        <v>179</v>
       </c>
       <c r="D53" s="13" t="s">
-        <v>140</v>
+        <v>131</v>
       </c>
       <c r="E53" s="13" t="s">
-        <v>198</v>
+        <v>189</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="13"/>
       <c r="B54" s="13"/>
       <c r="C54" s="13" t="s">
-        <v>199</v>
+        <v>190</v>
       </c>
       <c r="D54" s="13" t="s">
-        <v>140</v>
+        <v>131</v>
       </c>
       <c r="E54" s="13"/>
     </row>
@@ -2512,10 +2431,10 @@
       <c r="A55" s="13"/>
       <c r="B55" s="13"/>
       <c r="C55" s="13" t="s">
-        <v>200</v>
+        <v>191</v>
       </c>
       <c r="D55" s="13" t="s">
-        <v>140</v>
+        <v>131</v>
       </c>
       <c r="E55" s="13"/>
     </row>
@@ -2523,10 +2442,10 @@
       <c r="A56" s="13"/>
       <c r="B56" s="13"/>
       <c r="C56" s="13" t="s">
-        <v>154</v>
+        <v>145</v>
       </c>
       <c r="D56" s="13" t="s">
-        <v>155</v>
+        <v>146</v>
       </c>
       <c r="E56" s="13"/>
     </row>

</xml_diff>

<commit_message>
Plan rules UI after reference screens with first-match-wins rule lists
Rules now live in two ordered lists (checkout, post-order); the first
matching enabled rule is applied. Adds the full Filter Type catalog,
per-type match types, the Allow/Hold/Cancel action model and the
rules table and Add Rule page layouts. Estimate updated to 62.5h.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016VxfYAmeTkhYFto1GdTc34
</commit_message>
<xml_diff>
--- a/Store_Shield_Estimation.xlsx
+++ b/Store_Shield_Estimation.xlsx
@@ -37,7 +37,7 @@
     <t xml:space="preserve">Database setup and schema</t>
   </si>
   <si>
-    <t xml:space="preserve">Local PostgreSQL. Tables for settings, visits, rules, order checks, fraud list, staff actions and allowlist.</t>
+    <t xml:space="preserve">Local PostgreSQL with Prisma. Shop and settings tables; each later feature adds its own tables.</t>
   </si>
   <si>
     <t xml:space="preserve">App proxy and visitor check</t>
@@ -73,13 +73,13 @@
     <t xml:space="preserve">Rule engine core</t>
   </si>
   <si>
-    <t xml:space="preserve">Save rules and check their conditions with AND / OR. Live, test or off. Cancel wins over review when rules clash.</t>
+    <t xml:space="preserve">Two ordered rule lists (checkout and post-order). Check conditions with AND / OR. The first matching rule wins. Enable, disable, test mode, move up and down.</t>
   </si>
   <si>
     <t xml:space="preserve">Rule conditions</t>
   </si>
   <si>
-    <t xml:space="preserve">Cart value, products, address mismatch, postcode, country, disposable email, IP country, Shopify risk, repeat orders, past fraud.</t>
+    <t xml:space="preserve">All billing and shipping address fields, email, phone, name, order total and quantities, disposable email, chargebacks, Shopify risk and Protect, IP checks, repeat orders, same name/phone/address used by other customers, past fraud.</t>
   </si>
   <si>
     <t xml:space="preserve">Checkout function</t>
@@ -91,13 +91,13 @@
     <t xml:space="preserve">Order actions</t>
   </si>
   <si>
-    <t xml:space="preserve">When an order is placed: put it in review, auto-cancel (refund, restock, email customer), add tags, email the merchant.</t>
+    <t xml:space="preserve">Run the first matching rule: allow, hold fulfillment or cancel (refund, restock, notify customer), plus tag and email notification.</t>
   </si>
   <si>
     <t xml:space="preserve">Rules page and rule builder</t>
   </si>
   <si>
-    <t xml:space="preserve">List rules and turn them on or off. Builder to pick when, AND / OR, conditions and actions. Ready-made starter rules.</t>
+    <t xml:space="preserve">Rules table with list selector, search, chips, enable/disable, edit, delete and move up/down. Add Rule page with Rule Settings, Conditions and Actions cards. Starter rules.</t>
   </si>
   <si>
     <t xml:space="preserve">Orders page</t>
@@ -688,7 +688,7 @@
         <v>17</v>
       </c>
       <c r="D8" s="5" t="n">
-        <v>4</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -702,7 +702,7 @@
         <v>19</v>
       </c>
       <c r="D9" s="5" t="n">
-        <v>5</v>
+        <v>6.5</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -744,7 +744,7 @@
         <v>25</v>
       </c>
       <c r="D12" s="5" t="n">
-        <v>5.5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -825,7 +825,7 @@
       <c r="C18" s="6"/>
       <c r="D18" s="7" t="n">
         <f aca="false">SUM(D2:D17)</f>
-        <v>60</v>
+        <v>62.5</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>